<commit_message>
docs: fix test cases
</commit_message>
<xml_diff>
--- a/docs/ValidadorInversiones_PayFlow_EQ-NARANJA.xlsx
+++ b/docs/ValidadorInversiones_PayFlow_EQ-NARANJA.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OGSha\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA08E799-8C7B-4748-855D-DD35BD8F7B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40BAD793-4D8F-4DC9-9F45-558440FE6313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="20160" windowHeight="14295" xr2:uid="{88223292-B1B6-3447-BD61-E9A1A871A364}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{88223292-B1B6-3447-BD61-E9A1A871A364}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabla de Decisión" sheetId="1" r:id="rId1"/>
+    <sheet name="Tabla de Decisión Capa Inferior" sheetId="2" r:id="rId2"/>
+    <sheet name="Tabla de Decisión Capa Media" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,10 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="90">
-  <si>
-    <t>PRA05- Inversiones- PayFlow</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="107">
   <si>
     <t>Análisis para tabla de decisión</t>
   </si>
@@ -75,9 +74,6 @@
     <t>F</t>
   </si>
   <si>
-    <t>&lt;MONTO_FINAL_REDONDEADO&gt; [A=P(1+r)n]</t>
-  </si>
-  <si>
     <t>Mensajes (Errores/Notificación)</t>
   </si>
   <si>
@@ -186,18 +182,12 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>"Rechazada por ser cuenta nueva"</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
     <t>R</t>
   </si>
   <si>
-    <t>A=P(1+r)n</t>
-  </si>
-  <si>
     <t>"El plazo no puede ser menor a un año"</t>
   </si>
   <si>
@@ -295,13 +285,76 @@
   </si>
   <si>
     <t>AUTORIZADO[INVERSION_ESTABLE]</t>
+  </si>
+  <si>
+    <t>CONDICIONES/ACCIONES/ESCENARIOS</t>
+  </si>
+  <si>
+    <t>Bajo Riesgo</t>
+  </si>
+  <si>
+    <t>Alto Riesgo</t>
+  </si>
+  <si>
+    <t>Monto Negativo</t>
+  </si>
+  <si>
+    <t>Plazo Menor 1 Año</t>
+  </si>
+  <si>
+    <t>A=P(1+ r)^n</t>
+  </si>
+  <si>
+    <t>Inversión con bajo riesgo, monto negativo y plazo menor a 1 año</t>
+  </si>
+  <si>
+    <t>Inversión con bajo riesgo y monto negativo</t>
+  </si>
+  <si>
+    <t>Inversión con bajo riesgo y plazo menor a 1 año</t>
+  </si>
+  <si>
+    <t>Inversión con bajo riesgo</t>
+  </si>
+  <si>
+    <t>Inversión con alto riesgo, monto negativo y plazo menor a 1 año</t>
+  </si>
+  <si>
+    <t>Inversión con alto riesgo y monto negativo</t>
+  </si>
+  <si>
+    <t>Inversión con alto riesgo y plazo menor a 1 año</t>
+  </si>
+  <si>
+    <t>Inversión con alto riesgo</t>
+  </si>
+  <si>
+    <t>Tasa de Riesgo Anual (5% / 12%)</t>
+  </si>
+  <si>
+    <t>A=P(1 + r)^n</t>
+  </si>
+  <si>
+    <t>PRA05 - Inversiones- PayFlow</t>
+  </si>
+  <si>
+    <t>Análisis para Tabla de Decisión (Capa Inferior)</t>
+  </si>
+  <si>
+    <t>&lt;MONTO_FINAL_REDONDEADO&gt; [A=P(1+r)^n]</t>
+  </si>
+  <si>
+    <t>A=P(1+r)^n</t>
+  </si>
+  <si>
+    <t>Rechazada por exceder el saldo disponible</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -349,6 +402,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -388,7 +456,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -496,11 +564,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -589,6 +694,35 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -919,723 +1053,723 @@
   <sheetData>
     <row r="1" spans="1:34" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B1" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:34" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C2" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:34" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="29" t="s">
+      <c r="E3" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="29" t="s">
+      <c r="G3" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="30" t="s">
+      <c r="H3" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="I3" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="29" t="s">
+      <c r="J3" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="29" t="s">
+      <c r="O3" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="J3" s="21" t="s">
+      <c r="P3" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="O3" s="31" t="s">
+      <c r="Q3" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="P3" s="31" t="s">
+      <c r="R3" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="Q3" s="31" t="s">
+      <c r="S3" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="R3" s="32" t="s">
+      <c r="T3" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="S3" s="31" t="s">
+      <c r="U3" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="T3" s="31" t="s">
+      <c r="V3" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="U3" s="31" t="s">
+      <c r="W3" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="V3" s="31" t="s">
+      <c r="X3" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="W3" s="31" t="s">
+      <c r="Y3" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="X3" s="32" t="s">
+      <c r="Z3" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="Y3" s="31" t="s">
+      <c r="AE3" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="Z3" s="32" t="s">
+      <c r="AF3" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="AE3" s="31" t="s">
+      <c r="AG3" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="AF3" s="32" t="s">
+      <c r="AH3" s="32" t="s">
         <v>45</v>
-      </c>
-      <c r="AG3" s="31" t="s">
-        <v>46</v>
-      </c>
-      <c r="AH3" s="32" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:34" ht="96" x14ac:dyDescent="0.25">
       <c r="B4" s="6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C4" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="G4" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="H4" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="I4" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="J4" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="O4" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="P4" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q4" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="R4" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="S4" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="T4" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="U4" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="V4" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="W4" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="X4" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y4" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="Z4" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="AA4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="AC4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="AD4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="AE4" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="AF4" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="AG4" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="E4" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="F4" s="20" t="s">
+      <c r="AH4" s="24" t="s">
         <v>74</v>
-      </c>
-      <c r="G4" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="H4" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="I4" s="20" t="s">
-        <v>68</v>
-      </c>
-      <c r="J4" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="M4" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="N4" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="O4" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="P4" s="23" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q4" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="R4" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="S4" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="T4" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="U4" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="V4" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="W4" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="X4" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="Y4" s="23" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z4" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="AA4" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="AB4" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="AC4" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="AD4" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="AE4" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="AF4" s="24" t="s">
-        <v>79</v>
-      </c>
-      <c r="AG4" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="AH4" s="24" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:34" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N5" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O5" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q5" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="R5" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="S5" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="T5" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="U5" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="V5" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="W5" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="X5" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Y5" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Z5" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AA5" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AB5" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AC5" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AD5" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AE5" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AF5" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AG5" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AH5" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:34" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K6" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L6" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M6" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N6" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O6" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="P6" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q6" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="R6" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="T6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="U6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="V6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="W6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="X6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Y6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Z6" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AA6" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AB6" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AC6" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AD6" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AE6" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AF6" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AG6" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AH6" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:34" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K7" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L7" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M7" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N7" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="P7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="R7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S7" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="T7" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="V7" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="X7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Y7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Z7" s="14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AA7" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AB7" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AC7" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AD7" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AF7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AG7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AH7" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:34" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L8" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N8" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O8" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q8" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="R8" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S8" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="T8" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="U8" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="V8" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="W8" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="X8" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Y8" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Z8" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AA8" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AB8" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AC8" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AD8" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AE8" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AF8" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AG8" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AH8" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:34" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K9" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L9" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M9" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N9" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O9" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P9" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q9" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="R9" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="S9" s="7" t="s">
-        <v>14</v>
+        <v>14</v>
+      </c>
+      <c r="S9" s="34" t="s">
+        <v>13</v>
       </c>
       <c r="T9" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="U9" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="V9" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="W9" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="X9" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Y9" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Z9" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AA9" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AB9" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AC9" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AD9" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AE9" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AF9" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AG9" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AH9" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:34" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B14" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C14" s="16">
         <v>0.12</v>
@@ -1712,535 +1846,946 @@
     </row>
     <row r="15" spans="1:34" ht="110.25" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="J15" s="18" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="O15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="P15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="Q15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="R15" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="S15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="T15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="U15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="V15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="W15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="X15" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="Y15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="Z15" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="AE15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="AF15" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="AG15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="AH15" s="33" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:34" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="O16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="P16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="Q16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="R16" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="S16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="T16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="U16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="V16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="W16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="X16" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="Y16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="Z16" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="AE16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="AF16" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="AG16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="AH16" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="2:34" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C17" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="J17" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="O17" t="s">
+        <v>50</v>
+      </c>
+      <c r="P17" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>50</v>
+      </c>
+      <c r="R17" t="s">
+        <v>60</v>
+      </c>
+      <c r="S17" t="s">
+        <v>50</v>
+      </c>
+      <c r="T17" t="s">
+        <v>50</v>
+      </c>
+      <c r="U17" t="s">
+        <v>50</v>
+      </c>
+      <c r="V17" t="s">
+        <v>50</v>
+      </c>
+      <c r="W17" t="s">
+        <v>50</v>
+      </c>
+      <c r="X17" t="s">
         <v>52</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="Y17" t="s">
+        <v>50</v>
+      </c>
+      <c r="Z17" t="s">
         <v>52</v>
       </c>
-      <c r="F17" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="I17" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="J17" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="O17" t="s">
-        <v>52</v>
-      </c>
-      <c r="P17" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>52</v>
-      </c>
-      <c r="R17" t="s">
-        <v>64</v>
-      </c>
-      <c r="S17" t="s">
-        <v>52</v>
-      </c>
-      <c r="T17" t="s">
-        <v>52</v>
-      </c>
-      <c r="U17" t="s">
-        <v>52</v>
-      </c>
-      <c r="V17" t="s">
-        <v>52</v>
-      </c>
-      <c r="W17" t="s">
-        <v>52</v>
-      </c>
-      <c r="X17" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y17" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z17" t="s">
-        <v>55</v>
-      </c>
       <c r="AE17" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="AF17" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="AG17" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="AH17" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="2:34" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B18" s="5" t="s">
-        <v>16</v>
+        <v>104</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>56</v>
+        <v>105</v>
       </c>
       <c r="O18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="P18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="Q18" t="s">
-        <v>52</v>
-      </c>
-      <c r="R18" t="s">
-        <v>56</v>
+        <v>50</v>
+      </c>
+      <c r="R18" s="7" t="s">
+        <v>105</v>
       </c>
       <c r="S18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="T18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="U18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="V18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="W18" t="s">
-        <v>52</v>
-      </c>
-      <c r="X18" t="s">
-        <v>56</v>
+        <v>50</v>
+      </c>
+      <c r="X18" s="7" t="s">
+        <v>105</v>
       </c>
       <c r="Y18" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z18" t="s">
-        <v>56</v>
+        <v>50</v>
+      </c>
+      <c r="Z18" s="7" t="s">
+        <v>105</v>
       </c>
       <c r="AE18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="AF18" s="7" t="s">
-        <v>56</v>
+        <v>105</v>
       </c>
       <c r="AG18" t="s">
-        <v>52</v>
-      </c>
-      <c r="AH18" s="7" t="s">
-        <v>56</v>
+        <v>50</v>
+      </c>
+      <c r="AH18" s="46" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="2:34" ht="78.75" x14ac:dyDescent="0.25">
       <c r="B19" s="5" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="J19" s="26" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="K19" s="27"/>
       <c r="L19" s="27"/>
       <c r="M19" s="27"/>
       <c r="N19" s="27"/>
       <c r="O19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="P19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="Q19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="R19" s="15" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="S19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="T19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="U19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="V19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="W19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="X19" s="15" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="Y19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="Z19" s="15" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="AE19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="AF19" s="15" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="AG19" s="25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="AH19" s="15" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="2:34" ht="60.75" x14ac:dyDescent="0.25">
       <c r="B20" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="O20" s="15" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="P20" s="15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="Q20" s="15" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="R20" s="15"/>
       <c r="S20" s="15" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="T20" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="U20" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="V20" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="W20" s="15" t="s">
         <v>53</v>
       </c>
       <c r="X20" s="15"/>
       <c r="Y20" s="15" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="Z20" s="15"/>
       <c r="AE20" s="15" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="AF20" s="15"/>
       <c r="AG20" s="15" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="2:34" ht="60.75" x14ac:dyDescent="0.25">
       <c r="C21" s="15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="I21" s="15" t="s">
-        <v>58</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="I21" s="15"/>
       <c r="O21" s="15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="P21" s="15"/>
       <c r="Q21" s="15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="R21" s="15"/>
       <c r="S21" s="15" t="s">
-        <v>58</v>
+        <v>106</v>
       </c>
       <c r="U21" s="15" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="V21" s="15"/>
-      <c r="W21" s="15" t="s">
-        <v>58</v>
-      </c>
       <c r="X21" s="15"/>
-      <c r="Y21" s="15" t="s">
-        <v>58</v>
-      </c>
+      <c r="Y21" s="15"/>
       <c r="Z21" s="15"/>
       <c r="AE21" s="15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="AF21" s="15"/>
       <c r="AG21" s="15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="2:34" ht="60.75" x14ac:dyDescent="0.25">
       <c r="C22" s="15" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D22" s="15"/>
-      <c r="E22" s="15" t="s">
-        <v>58</v>
-      </c>
+      <c r="E22" s="15"/>
       <c r="G22" s="15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="O22" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="S22" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="U22" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="W22" s="15" t="s">
-        <v>57</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="S22" s="15"/>
       <c r="Y22" s="15"/>
     </row>
-    <row r="23" spans="2:34" ht="48.75" x14ac:dyDescent="0.25">
-      <c r="C23" s="15" t="s">
-        <v>58</v>
-      </c>
+    <row r="23" spans="2:34" x14ac:dyDescent="0.25">
+      <c r="C23" s="15"/>
       <c r="D23" s="15"/>
+      <c r="E23" s="33"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2497A194-E15B-4A64-9F4A-CF0D4BC9116E}">
+  <dimension ref="A1:Q14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.875" customWidth="1"/>
+    <col min="2" max="5" width="11" style="11"/>
+    <col min="6" max="6" width="12.75" customWidth="1"/>
+    <col min="14" max="17" width="11" style="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F2" s="44" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="26.25" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F3" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="40" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="41" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" s="40" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" s="40" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" s="40" t="s">
+        <v>28</v>
+      </c>
+      <c r="M3" s="42" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="A4" s="43" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="G4" s="45" t="s">
+        <v>93</v>
+      </c>
+      <c r="H4" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="I4" s="38" t="s">
+        <v>95</v>
+      </c>
+      <c r="J4" s="37" t="s">
+        <v>96</v>
+      </c>
+      <c r="K4" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="L4" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="M4" s="38" t="s">
+        <v>99</v>
+      </c>
+      <c r="N4" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="O4" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="P4" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q4" s="36" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="L5" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="M5" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="N5" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="O5" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="P5" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q5" s="36" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="K6" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="L6" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="M6" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="N6" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="O6" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="P6" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q6" s="36" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="I7" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="L7" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="M7" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="N7" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="O7" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="P7" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q7" s="36" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="L8" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="M8" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="N8" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="O8" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="P8" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q8" s="36" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" s="43" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="F11" s="22">
+        <v>0.05</v>
+      </c>
+      <c r="G11" s="22">
+        <v>0.05</v>
+      </c>
+      <c r="H11" s="22">
+        <v>0.05</v>
+      </c>
+      <c r="I11" s="22">
+        <v>0.05</v>
+      </c>
+      <c r="J11" s="22">
+        <v>0.12</v>
+      </c>
+      <c r="K11" s="22">
+        <v>0.12</v>
+      </c>
+      <c r="L11" s="22">
+        <v>0.12</v>
+      </c>
+      <c r="M11" s="22">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>91</v>
+      </c>
+      <c r="F12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G12" t="s">
+        <v>50</v>
+      </c>
+      <c r="H12" t="s">
+        <v>50</v>
+      </c>
+      <c r="I12" t="s">
+        <v>91</v>
+      </c>
+      <c r="J12" t="s">
+        <v>50</v>
+      </c>
+      <c r="K12" t="s">
+        <v>50</v>
+      </c>
+      <c r="L12" t="s">
+        <v>50</v>
+      </c>
+      <c r="M12" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="48.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="J13" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="K13" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="L13" s="15" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="48.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="5"/>
+      <c r="F14" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="H14" s="15"/>
+      <c r="J14" s="15" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCCB26C9-2881-49A8-96E8-A4D4477D580A}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>